<commit_message>
Day 3 load counts and match GSM sample IDs
</commit_message>
<xml_diff>
--- a/metadata/sample_metadata.xlsx
+++ b/metadata/sample_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devarshdesai/Desktop/Bioinformatics_Career/02_Projects/crc-bulk-rnaseq-deseq1/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3687C544-A919-2040-B4CC-8BD374558909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1EB65F-9BCE-8A49-8DB6-DF36F672BCDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28800" yWindow="2300" windowWidth="21600" windowHeight="15700" xr2:uid="{996B531E-1639-604F-B637-4931523715D9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="111">
   <si>
     <t>sample_id</t>
   </si>
@@ -306,6 +306,69 @@
   </si>
   <si>
     <t>colorectal tumor tissue</t>
+  </si>
+  <si>
+    <t>gsm_id</t>
+  </si>
+  <si>
+    <t>RC1</t>
+  </si>
+  <si>
+    <t>RC2</t>
+  </si>
+  <si>
+    <t>RC3</t>
+  </si>
+  <si>
+    <t>RC4</t>
+  </si>
+  <si>
+    <t>RC5</t>
+  </si>
+  <si>
+    <t>RC6</t>
+  </si>
+  <si>
+    <t>LC1</t>
+  </si>
+  <si>
+    <t>LC2</t>
+  </si>
+  <si>
+    <t>LC3</t>
+  </si>
+  <si>
+    <t>LC4</t>
+  </si>
+  <si>
+    <t>LC5</t>
+  </si>
+  <si>
+    <t>LC6</t>
+  </si>
+  <si>
+    <t>RE1</t>
+  </si>
+  <si>
+    <t>RE2</t>
+  </si>
+  <si>
+    <t>RE3</t>
+  </si>
+  <si>
+    <t>RE4</t>
+  </si>
+  <si>
+    <t>RE5</t>
+  </si>
+  <si>
+    <t>RE6</t>
+  </si>
+  <si>
+    <t>RE7</t>
+  </si>
+  <si>
+    <t>RE8</t>
   </si>
 </sst>
 </file>
@@ -410,11 +473,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -431,6 +491,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -768,14 +834,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{381F6ED8-F9F9-294E-9257-86189448ADC8}">
-  <dimension ref="B2:G42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="14.1640625" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A2:G42"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="18.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>90</v>
+      </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -788,35 +853,41 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B3" s="3" t="s">
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B4" s="3" t="s">
+      <c r="F3" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>91</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>86</v>
@@ -824,35 +895,41 @@
       <c r="E4" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B5" s="3" t="s">
+      <c r="F4" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="F5" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G5" s="6"/>
+    </row>
+    <row r="6" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="C6" s="1" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>86</v>
@@ -860,35 +937,41 @@
       <c r="E6" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="F6" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="C7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B8" s="3" t="s">
+      <c r="F7" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="6"/>
+    </row>
+    <row r="8" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="B8" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="C8" s="1" t="s">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>86</v>
@@ -896,35 +979,41 @@
       <c r="E8" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8" s="7"/>
-    </row>
-    <row r="9" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B9" s="3" t="s">
+      <c r="F8" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="6"/>
+    </row>
+    <row r="9" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B10" s="3" t="s">
+      <c r="F9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="B10" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>94</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>86</v>
@@ -932,35 +1021,41 @@
       <c r="E10" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G10" s="7"/>
-    </row>
-    <row r="11" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B11" s="3" t="s">
+      <c r="F10" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="B11" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="C11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B12" s="3" t="s">
+      <c r="F11" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G11" s="6"/>
+    </row>
+    <row r="12" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="B12" s="1" t="s">
+        <v>24</v>
+      </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>86</v>
@@ -968,17 +1063,20 @@
       <c r="E12" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F12" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B13" s="3" t="s">
+      <c r="F12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="B13" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="C13" s="1" t="s">
-        <v>26</v>
+        <v>96</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>85</v>
@@ -986,17 +1084,20 @@
       <c r="E13" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G13" s="7"/>
-    </row>
-    <row r="14" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B14" s="3" t="s">
+      <c r="F13" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="B14" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="C14" s="1" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>86</v>
@@ -1004,35 +1105,41 @@
       <c r="E14" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G14" s="7"/>
-    </row>
-    <row r="15" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B15" s="3" t="s">
+      <c r="F14" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="B15" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="C15" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G15" s="7"/>
-    </row>
-    <row r="16" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B16" s="3" t="s">
+      <c r="F15" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="B16" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="C16" s="1" t="s">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>86</v>
@@ -1040,35 +1147,41 @@
       <c r="E16" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G16" s="7"/>
-    </row>
-    <row r="17" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B17" s="3" t="s">
+      <c r="F16" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>33</v>
       </c>
+      <c r="B17" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="C17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G17" s="7"/>
-    </row>
-    <row r="18" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B18" s="3" t="s">
+      <c r="F17" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="B18" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="C18" s="1" t="s">
-        <v>36</v>
+        <v>98</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>86</v>
@@ -1076,35 +1189,41 @@
       <c r="E18" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="7"/>
-    </row>
-    <row r="19" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B19" s="3" t="s">
+      <c r="F18" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>37</v>
       </c>
+      <c r="B19" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="C19" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G19" s="7"/>
-    </row>
-    <row r="20" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B20" s="3" t="s">
+      <c r="F19" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
+      <c r="B20" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="C20" s="1" t="s">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>86</v>
@@ -1112,35 +1231,41 @@
       <c r="E20" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G20" s="7"/>
-    </row>
-    <row r="21" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B21" s="3" t="s">
+      <c r="F20" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="B21" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="C21" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G21" s="7"/>
-    </row>
-    <row r="22" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B22" s="3" t="s">
+      <c r="F21" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
+      <c r="B22" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="C22" s="1" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>86</v>
@@ -1148,35 +1273,41 @@
       <c r="E22" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G22" s="7"/>
-    </row>
-    <row r="23" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B23" s="3" t="s">
+      <c r="F22" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>45</v>
       </c>
+      <c r="B23" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="C23" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D23" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23" s="7"/>
-    </row>
-    <row r="24" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B24" s="3" t="s">
+      <c r="F23" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
+      <c r="B24" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="C24" s="1" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>86</v>
@@ -1184,35 +1315,41 @@
       <c r="E24" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G24" s="7"/>
-    </row>
-    <row r="25" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B25" s="3" t="s">
+      <c r="F24" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>49</v>
       </c>
+      <c r="B25" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="C25" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D25" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G25" s="7"/>
-    </row>
-    <row r="26" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B26" s="3" t="s">
+      <c r="F25" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
       <c r="C26" s="1" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>86</v>
@@ -1220,35 +1357,41 @@
       <c r="E26" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G26" s="7"/>
-    </row>
-    <row r="27" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B27" s="3" t="s">
+      <c r="F26" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="27" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="B27" s="1" t="s">
+        <v>54</v>
+      </c>
       <c r="C27" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D27" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G27" s="7"/>
-    </row>
-    <row r="28" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B28" s="3" t="s">
+      <c r="F27" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="28" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>55</v>
       </c>
+      <c r="B28" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="C28" s="1" t="s">
-        <v>56</v>
+        <v>103</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>86</v>
@@ -1256,35 +1399,41 @@
       <c r="E28" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G28" s="7"/>
-    </row>
-    <row r="29" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B29" s="3" t="s">
+      <c r="F28" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>57</v>
       </c>
+      <c r="B29" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="C29" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D29" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G29" s="7"/>
-    </row>
-    <row r="30" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B30" s="3" t="s">
+      <c r="F29" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G29" s="6"/>
+    </row>
+    <row r="30" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>59</v>
       </c>
+      <c r="B30" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="C30" s="1" t="s">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>86</v>
@@ -1292,35 +1441,41 @@
       <c r="E30" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G30" s="7"/>
-    </row>
-    <row r="31" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B31" s="3" t="s">
+      <c r="F30" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G30" s="6"/>
+    </row>
+    <row r="31" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="B31" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="C31" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G31" s="7"/>
-    </row>
-    <row r="32" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B32" s="3" t="s">
+      <c r="F31" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G31" s="6"/>
+    </row>
+    <row r="32" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>63</v>
       </c>
+      <c r="B32" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="C32" s="1" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>86</v>
@@ -1328,35 +1483,41 @@
       <c r="E32" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G32" s="7"/>
-    </row>
-    <row r="33" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B33" s="3" t="s">
+      <c r="F32" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>65</v>
       </c>
+      <c r="B33" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="C33" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D33" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D33" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G33" s="7"/>
-    </row>
-    <row r="34" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B34" s="3" t="s">
+      <c r="F33" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>67</v>
       </c>
+      <c r="B34" s="1" t="s">
+        <v>68</v>
+      </c>
       <c r="C34" s="1" t="s">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>86</v>
@@ -1364,35 +1525,41 @@
       <c r="E34" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G34" s="7"/>
-    </row>
-    <row r="35" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B35" s="3" t="s">
+      <c r="F34" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G34" s="6"/>
+    </row>
+    <row r="35" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>69</v>
       </c>
+      <c r="B35" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="C35" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D35" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G35" s="7"/>
-    </row>
-    <row r="36" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B36" s="3" t="s">
+      <c r="F35" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>71</v>
       </c>
+      <c r="B36" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="C36" s="1" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>86</v>
@@ -1400,35 +1567,41 @@
       <c r="E36" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F36" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G36" s="7"/>
-    </row>
-    <row r="37" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B37" s="3" t="s">
+      <c r="F36" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>73</v>
       </c>
+      <c r="B37" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="C37" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D37" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G37" s="7"/>
-    </row>
-    <row r="38" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B38" s="3" t="s">
+      <c r="F37" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>75</v>
       </c>
+      <c r="B38" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="C38" s="1" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>86</v>
@@ -1436,35 +1609,41 @@
       <c r="E38" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F38" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G38" s="7"/>
-    </row>
-    <row r="39" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B39" s="3" t="s">
+      <c r="F38" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G38" s="6"/>
+    </row>
+    <row r="39" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>77</v>
       </c>
+      <c r="B39" s="1" t="s">
+        <v>78</v>
+      </c>
       <c r="C39" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D39" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D39" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G39" s="7"/>
-    </row>
-    <row r="40" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B40" s="3" t="s">
+      <c r="F39" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G39" s="6"/>
+    </row>
+    <row r="40" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>79</v>
       </c>
+      <c r="B40" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="C40" s="1" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>86</v>
@@ -1472,35 +1651,41 @@
       <c r="E40" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F40" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G40" s="7"/>
-    </row>
-    <row r="41" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B41" s="3" t="s">
+      <c r="F40" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>81</v>
       </c>
+      <c r="B41" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="C41" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D41" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" s="4" t="s">
         <v>85</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F41" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="G41" s="7"/>
-    </row>
-    <row r="42" spans="2:7" ht="18" x14ac:dyDescent="0.2">
-      <c r="B42" s="3" t="s">
+      <c r="F41" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>83</v>
       </c>
+      <c r="B42" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="C42" s="1" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>86</v>
@@ -1508,13 +1693,46 @@
       <c r="E42" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G42" s="7"/>
+      <c r="F42" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G42" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="F42:G42"/>
     <mergeCell ref="F35:G35"/>
@@ -1523,80 +1741,47 @@
     <mergeCell ref="F38:G38"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224324" xr:uid="{1385642F-4FCC-6C41-92EF-454799DEC23F}"/>
-    <hyperlink ref="B5" r:id="rId2" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224325" xr:uid="{8DA59126-E366-8A4D-8B4B-AB146E61EE2B}"/>
-    <hyperlink ref="B6" r:id="rId3" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224326" xr:uid="{D7F58E64-BA3F-BC4B-B71C-1F3DF2D55B56}"/>
-    <hyperlink ref="B7" r:id="rId4" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224327" xr:uid="{3970D30C-9729-A845-848D-DDEC5ED44047}"/>
-    <hyperlink ref="B8" r:id="rId5" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224328" xr:uid="{16AFF089-8167-AE4D-8ADD-C379DC949F2D}"/>
-    <hyperlink ref="B9" r:id="rId6" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224329" xr:uid="{B1F1C590-2012-F04D-86CB-6EB42F0F4C64}"/>
-    <hyperlink ref="B10" r:id="rId7" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224330" xr:uid="{9C19D38D-6343-5240-9D43-D483EF4CFAD7}"/>
-    <hyperlink ref="B11" r:id="rId8" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224331" xr:uid="{C3080128-178F-9743-B302-ABE915E725C0}"/>
-    <hyperlink ref="B12" r:id="rId9" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224332" xr:uid="{0DF9A607-2A51-ED47-9CD7-95C8493C4F31}"/>
-    <hyperlink ref="B13" r:id="rId10" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224333" xr:uid="{30421870-2548-FB42-A896-B1A31CFB9294}"/>
-    <hyperlink ref="B14" r:id="rId11" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224334" xr:uid="{F6DDD084-5554-A34E-88EC-09550A11F7CD}"/>
-    <hyperlink ref="B15" r:id="rId12" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224335" xr:uid="{57E0C73D-72F2-4D43-AD59-8A3ED16D6F8B}"/>
-    <hyperlink ref="B16" r:id="rId13" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224336" xr:uid="{2D25E33C-A01E-DF41-BB98-7588AAE86497}"/>
-    <hyperlink ref="B17" r:id="rId14" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224337" xr:uid="{36BA1521-C8C9-6C45-890B-EB1D5778B092}"/>
-    <hyperlink ref="B18" r:id="rId15" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224338" xr:uid="{340EF4D8-4A0D-BD44-8346-B80728A638B9}"/>
-    <hyperlink ref="B19" r:id="rId16" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224339" xr:uid="{92FBCA2C-3F5F-924F-BA91-25E3ADB35BD9}"/>
-    <hyperlink ref="B20" r:id="rId17" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224340" xr:uid="{65711EBC-98F8-3D44-8DE0-7DFBE1368BF2}"/>
-    <hyperlink ref="B21" r:id="rId18" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224341" xr:uid="{BF78334F-4F1D-A74D-A33C-B82569990709}"/>
-    <hyperlink ref="B22" r:id="rId19" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224342" xr:uid="{E33DF0C3-B414-B546-A851-B8741E7A1963}"/>
-    <hyperlink ref="B23" r:id="rId20" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224343" xr:uid="{56BB6CF0-73CD-974A-A1E5-4A721D8B61C6}"/>
-    <hyperlink ref="B24" r:id="rId21" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224344" xr:uid="{A07DE339-BA15-8C47-82BC-A55D05328298}"/>
-    <hyperlink ref="B25" r:id="rId22" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224345" xr:uid="{45768953-D929-E649-B993-5B38E816E5DF}"/>
-    <hyperlink ref="B26" r:id="rId23" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224346" xr:uid="{442B9408-BE77-7B49-8467-A5A10A971CD3}"/>
-    <hyperlink ref="B27" r:id="rId24" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224347" xr:uid="{199AE74F-657A-6245-9A3C-32AA9ED37C5C}"/>
-    <hyperlink ref="B28" r:id="rId25" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224348" xr:uid="{72881501-A782-DF47-954F-E15EF51F5E3E}"/>
-    <hyperlink ref="B29" r:id="rId26" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224349" xr:uid="{D0046292-37BA-F646-86D0-C5B7A1026345}"/>
-    <hyperlink ref="B30" r:id="rId27" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224350" xr:uid="{FDDD7D29-A98E-174B-A54E-7BC869DFDB81}"/>
-    <hyperlink ref="B31" r:id="rId28" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224351" xr:uid="{BBDF93C8-4768-274F-9566-E740C9857F73}"/>
-    <hyperlink ref="B32" r:id="rId29" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224352" xr:uid="{73E02D5A-B3F8-3D4E-97DC-F49357CF5EFF}"/>
-    <hyperlink ref="B33" r:id="rId30" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224353" xr:uid="{396DFEDB-C33C-B143-9F73-8D8D1C910A51}"/>
-    <hyperlink ref="B34" r:id="rId31" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224354" xr:uid="{DEEB93FF-A660-704E-98DD-CC619C84C38C}"/>
-    <hyperlink ref="B35" r:id="rId32" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224355" xr:uid="{2A61C22D-CD13-A649-B078-44CB154B5EFB}"/>
-    <hyperlink ref="B36" r:id="rId33" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224356" xr:uid="{1919F278-AFD2-9F4F-AD31-77C9EF2A7759}"/>
-    <hyperlink ref="B37" r:id="rId34" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224357" xr:uid="{265CC4B2-B0D4-1D48-8C9B-B31ADC027049}"/>
-    <hyperlink ref="B38" r:id="rId35" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224358" xr:uid="{665AAED3-2017-7847-88A5-FB4D586E196C}"/>
-    <hyperlink ref="B39" r:id="rId36" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224359" xr:uid="{FCD54F7B-50D8-CB47-9CAF-5E4594AAA05E}"/>
-    <hyperlink ref="B40" r:id="rId37" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224360" xr:uid="{44E82137-C105-5246-B84D-8CC840535C42}"/>
-    <hyperlink ref="B41" r:id="rId38" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224361" xr:uid="{346D4B4F-0308-F248-917E-F788EE11A68E}"/>
-    <hyperlink ref="B42" r:id="rId39" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224362" xr:uid="{E4C51715-B83D-7E47-BF4C-5B443DB8CD5E}"/>
+    <hyperlink ref="A4" r:id="rId1" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224324" xr:uid="{AEB20ACC-9B0B-7C48-BAE4-512A01C5D573}"/>
+    <hyperlink ref="A5" r:id="rId2" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224325" xr:uid="{90CE9452-BB9A-5047-A6EC-6ED054C8C396}"/>
+    <hyperlink ref="A6" r:id="rId3" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224326" xr:uid="{97AFC80A-53E6-1C4E-A98B-9051A342C4AC}"/>
+    <hyperlink ref="A7" r:id="rId4" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224327" xr:uid="{3DB30BFF-CE46-BB4D-9464-2578D9FF259D}"/>
+    <hyperlink ref="A8" r:id="rId5" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224328" xr:uid="{37E921BF-B42D-D046-B193-02C97D4545A2}"/>
+    <hyperlink ref="A9" r:id="rId6" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224329" xr:uid="{D991F418-D298-4741-91A4-895FB928203F}"/>
+    <hyperlink ref="A10" r:id="rId7" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224330" xr:uid="{30D423FF-1712-BC46-AD89-9F1E4F495F8A}"/>
+    <hyperlink ref="A11" r:id="rId8" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224331" xr:uid="{A0C48774-9B47-8D4F-AF17-CE04994DB466}"/>
+    <hyperlink ref="A12" r:id="rId9" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224332" xr:uid="{9B5F404C-6AFF-0A45-8781-5A493CD2C53E}"/>
+    <hyperlink ref="A13" r:id="rId10" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224333" xr:uid="{C07C0852-4FF2-7F42-959F-DB2A0D456431}"/>
+    <hyperlink ref="A14" r:id="rId11" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224334" xr:uid="{B571E6AA-F338-E04F-A39F-19FCF860AD27}"/>
+    <hyperlink ref="A15" r:id="rId12" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224335" xr:uid="{A01AB22F-FB4F-4547-9158-541D919EF26E}"/>
+    <hyperlink ref="A16" r:id="rId13" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224336" xr:uid="{459E1DBE-E49A-3841-86CC-CDFC06B5E3D6}"/>
+    <hyperlink ref="A17" r:id="rId14" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224337" xr:uid="{36D28ECB-B148-FA4B-95F2-058EA8C46626}"/>
+    <hyperlink ref="A18" r:id="rId15" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224338" xr:uid="{8F07D22F-F47C-A44D-B4B6-4ADD8E8879A2}"/>
+    <hyperlink ref="A19" r:id="rId16" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224339" xr:uid="{8392745C-E4B9-C948-BF16-74C31F91E378}"/>
+    <hyperlink ref="A20" r:id="rId17" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224340" xr:uid="{04C6059A-E0DC-294E-9E80-122019E75C50}"/>
+    <hyperlink ref="A21" r:id="rId18" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224341" xr:uid="{12788D67-DD97-FA43-A7E0-80B2DAC15CD2}"/>
+    <hyperlink ref="A22" r:id="rId19" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224342" xr:uid="{087987D5-8A30-7B4A-9AE1-EBF79E86CFBC}"/>
+    <hyperlink ref="A23" r:id="rId20" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224343" xr:uid="{6311F220-FC6A-FB48-A4AE-D2A9B086CF54}"/>
+    <hyperlink ref="A24" r:id="rId21" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224344" xr:uid="{A3D1650E-9C59-2F4C-8EE1-A98318A45B6E}"/>
+    <hyperlink ref="A25" r:id="rId22" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224345" xr:uid="{ACD7DCB4-4743-1945-AF12-55F9993305FA}"/>
+    <hyperlink ref="A26" r:id="rId23" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224346" xr:uid="{CAC331BE-471C-8B43-93F8-33DFD8413929}"/>
+    <hyperlink ref="A27" r:id="rId24" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224347" xr:uid="{19199CAA-2528-CE4C-8E91-46AB63073ADA}"/>
+    <hyperlink ref="A28" r:id="rId25" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224348" xr:uid="{7143155D-54BB-D64E-9BA0-724C9A4D0D27}"/>
+    <hyperlink ref="A29" r:id="rId26" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224349" xr:uid="{00B10B8B-F1A5-CD41-B9D0-6C3B92915C85}"/>
+    <hyperlink ref="A30" r:id="rId27" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224350" xr:uid="{D4C2C05F-95D1-874E-9655-C001766916D5}"/>
+    <hyperlink ref="A31" r:id="rId28" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224351" xr:uid="{F372F242-FEF0-234D-86F6-C1A548BCA279}"/>
+    <hyperlink ref="A32" r:id="rId29" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224352" xr:uid="{51FDDBA8-E08C-9142-8345-9875896E658F}"/>
+    <hyperlink ref="A33" r:id="rId30" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224353" xr:uid="{8EAD9CC4-666E-FE4B-A4BE-65A6DDE669A5}"/>
+    <hyperlink ref="A34" r:id="rId31" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224354" xr:uid="{9D8428F9-568F-BA41-AA7E-2886FF23A0C5}"/>
+    <hyperlink ref="A35" r:id="rId32" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224355" xr:uid="{6CA3B7BF-85D6-174E-8806-F3AE72D5C9FC}"/>
+    <hyperlink ref="A36" r:id="rId33" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224356" xr:uid="{5E962E4D-7D41-584E-B29E-AE90F9E3E39F}"/>
+    <hyperlink ref="A37" r:id="rId34" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224357" xr:uid="{736ABAD9-4EC9-E848-AC30-F37FB0E4D29A}"/>
+    <hyperlink ref="A38" r:id="rId35" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224358" xr:uid="{B996761F-ED4F-6E46-B96F-8AEDC3FFF281}"/>
+    <hyperlink ref="A39" r:id="rId36" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224359" xr:uid="{1A6D4D0A-4E29-7647-8327-4E068F499D47}"/>
+    <hyperlink ref="A40" r:id="rId37" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224360" xr:uid="{4A9D5F5D-3CA3-1640-8BC9-0C7AA2603042}"/>
+    <hyperlink ref="A41" r:id="rId38" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224361" xr:uid="{E3E2A7F7-AF3D-2747-8845-20A94FD8ED9F}"/>
+    <hyperlink ref="A42" r:id="rId39" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM4224362" xr:uid="{BC4D264E-A3AC-254C-A2F4-9B67B580B1A9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>